<commit_message>
Prepare SP2I cloud deployment and cockpit
</commit_message>
<xml_diff>
--- a/05_RESULTATS/audit_qualite_dqe.xlsx
+++ b/05_RESULTATS/audit_qualite_dqe.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,32 +466,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DQE-000067</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aucune anomalie critique</t>
+          <t>Baie vitrée en alu 220x90</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>menuiserie</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>COMMUN_BATIMENT</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -502,7 +502,136 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DQE-000068</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Baie vitrée en alu 220x80</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>menuiserie</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>COMMUN_BATIMENT</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DQE-000076</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Baie vitrée en alu 220x90</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>menuiserie</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>COMMUN_BATIMENT</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DQE-000077</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Baie vitrée en alu 220x80</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>menuiserie</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>COMMUN_BATIMENT</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(dqe): use normalized row count for enterprise preview
</commit_message>
<xml_diff>
--- a/05_RESULTATS/audit_qualite_dqe.xlsx
+++ b/05_RESULTATS/audit_qualite_dqe.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,27 +466,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DQE-000067</t>
+          <t>OBJ_SOL_001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Baie vitrée en alu 220x90</t>
+          <t>Panneaux photovoltaïques</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
+          <t>LOT_SOL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>menuiserie</t>
+          <t>plomberie</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>TOITURE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,143 +495,14 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DQE-000068</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Baie vitrée en alu 220x80</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>menuiserie</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>COMMUN_BATIMENT</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DQE-000076</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Baie vitrée en alu 220x90</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>menuiserie</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>COMMUN_BATIMENT</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DQE-000077</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Baie vitrée en alu 220x80</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>LOT 4 : MENUISERIE ALUMINIUM ET VITRERIE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>menuiserie</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>COMMUN_BATIMENT</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>QUANTITE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
+          <t>PRIX_UNITAIRE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restore analytics consistency and synchronize dashboard with FACT_METRE
</commit_message>
<xml_diff>
--- a/05_RESULTATS/audit_qualite_dqe.xlsx
+++ b/05_RESULTATS/audit_qualite_dqe.xlsx
@@ -466,43 +466,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OBJ_SOL_001</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Panneaux photovoltaïques</t>
+          <t>Aucune anomalie critique</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LOT_SOL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>plomberie</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TOITURE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>COMMUN_BATIMENT</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>PRIX_UNITAIRE_INVALIDE|PRIX_TOTAL_INVALIDE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>

</xml_diff>